<commit_message>
Update BOMs to replace voltage regulator
</commit_message>
<xml_diff>
--- a/schematics/Uzebox-Omega/V1.1.1/Uzebox-Omega-1.1.1-BOM-DigiKey.xlsx
+++ b/schematics/Uzebox-Omega/V1.1.1/Uzebox-Omega-1.1.1-BOM-DigiKey.xlsx
@@ -28,40 +28,7 @@
     <t xml:space="preserve">Quantity</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Tahoma"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Uzebox Omega v1.1.1 Digi-Key BOM. Last updated 5</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <vertAlign val="superscript"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Tahoma"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">th</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Tahoma"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> September 2025.</t>
-    </r>
+    <t xml:space="preserve">Uzebox Omega v1.1.1 Digi-Key BOM. Last updated 12th February 2026.</t>
   </si>
   <si>
     <t xml:space="preserve">2092-KMDGX-9S-N-ND</t>
@@ -178,10 +145,10 @@
     <t xml:space="preserve">IC MCU AVR 64K FLASH 40-DIP         (MCU)</t>
   </si>
   <si>
-    <t xml:space="preserve">MC7805ACTGOS-ND</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IC REG POS 1A 5V                    (IC2)</t>
+    <t xml:space="preserve">497-1443-5-ND</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IC REG LINEAR 5V 1.5A TO220                    (IC2)</t>
   </si>
   <si>
     <t xml:space="preserve">641-1310-1-ND</t>
@@ -227,7 +194,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -260,15 +227,6 @@
     </font>
     <font>
       <b val="true"/>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Tahoma"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <vertAlign val="superscript"/>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Tahoma"/>
@@ -425,7 +383,7 @@
   <dimension ref="A1:C27"/>
   <sheetFormatPr defaultColWidth="8.42578125" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="23.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="23.39"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="144.34"/>
   </cols>

</xml_diff>

<commit_message>
Change mini DIN socket part for DigiKey BOM
</commit_message>
<xml_diff>
--- a/schematics/Uzebox-Omega/V1.1.1/Uzebox-Omega-1.1.1-BOM-DigiKey.xlsx
+++ b/schematics/Uzebox-Omega/V1.1.1/Uzebox-Omega-1.1.1-BOM-DigiKey.xlsx
@@ -28,10 +28,10 @@
     <t xml:space="preserve">Quantity</t>
   </si>
   <si>
-    <t xml:space="preserve">Uzebox Omega v1.1.1 Digi-Key BOM. Last updated 26th April 2026.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2092-KMDGX-9S-N-ND</t>
+    <t xml:space="preserve">Uzebox Omega v1.1.1 Digi-Key BOM. Last updated 9th August 2026.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2092-KMDGX-9S-BS-1-ND</t>
   </si>
   <si>
     <t xml:space="preserve">CONN RCPT FMALE MINI DIN 9P SLDR   (X1)</t>
@@ -112,7 +112,7 @@
     <t xml:space="preserve">562XBK-ND</t>
   </si>
   <si>
-    <t xml:space="preserve">RES 562 OHM 1/4W 1% METAL FILM      (R29,R30,R31) and video fix</t>
+    <t xml:space="preserve">RES 562 OHM 1/4W 1% METAL FILM      (R29,R30,R31) and X1 video fix</t>
   </si>
   <si>
     <t xml:space="preserve">3.16KXBK-ND</t>
@@ -381,7 +381,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C27"/>
-  <sheetFormatPr defaultColWidth="8.42578125" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.43359375" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="23.4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="9"/>

</xml_diff>